<commit_message>
Update website chapters and draft assets
</commit_message>
<xml_diff>
--- a/docs/results/ch2_fw1_rotated_loading_table.xlsx
+++ b/docs/results/ch2_fw1_rotated_loading_table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,11 +464,6 @@
           <t>PC6</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>PC7</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -477,25 +472,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6772</v>
+        <v>0.76354</v>
       </c>
       <c r="C2" t="n">
-        <v>0.65832</v>
+        <v>0.45655</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0279</v>
+        <v>0.00615</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06877</v>
+        <v>0.07246</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1882</v>
+        <v>0.34743</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06371</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.05711</v>
+        <v>0.06092</v>
       </c>
     </row>
     <row r="3">
@@ -505,25 +497,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.46094</v>
+        <v>0.56757</v>
       </c>
       <c r="C3" t="n">
-        <v>0.80847</v>
+        <v>0.67184</v>
       </c>
       <c r="D3" t="n">
-        <v>0.04369</v>
+        <v>0.007889999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02137</v>
+        <v>0.03446</v>
       </c>
       <c r="F3" t="n">
-        <v>0.11183</v>
+        <v>0.32983</v>
       </c>
       <c r="G3" t="n">
-        <v>0.14044</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.18617</v>
+        <v>0.18482</v>
       </c>
     </row>
     <row r="4">
@@ -533,25 +522,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.8861</v>
+        <v>0.88186</v>
       </c>
       <c r="C4" t="n">
-        <v>0.01934</v>
+        <v>-0.04351</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.02909</v>
+        <v>-0.06543</v>
       </c>
       <c r="E4" t="n">
-        <v>0.03109</v>
+        <v>0.03855</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.26362</v>
+        <v>-0.27557</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.00202</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.11859</v>
+        <v>0.06308999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -561,25 +547,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.50124</v>
+        <v>0.58973</v>
       </c>
       <c r="C5" t="n">
-        <v>0.38599</v>
+        <v>0.41491</v>
       </c>
       <c r="D5" t="n">
-        <v>0.36654</v>
+        <v>0.30513</v>
       </c>
       <c r="E5" t="n">
-        <v>0.15394</v>
+        <v>0.16302</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.37012</v>
+        <v>-0.26725</v>
       </c>
       <c r="G5" t="n">
-        <v>0.15851</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.38914</v>
+        <v>0.38352</v>
       </c>
     </row>
     <row r="6">
@@ -589,25 +572,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4722</v>
+        <v>0.79231</v>
       </c>
       <c r="C6" t="n">
-        <v>0.17118</v>
+        <v>0.16983</v>
       </c>
       <c r="D6" t="n">
-        <v>0.05791</v>
+        <v>0.02921</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0212</v>
+        <v>0.02446</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01899</v>
+        <v>0.05188</v>
       </c>
       <c r="G6" t="n">
-        <v>0.84202</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.14146</v>
+        <v>0.23469</v>
       </c>
     </row>
     <row r="7">
@@ -617,25 +597,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.91736</v>
+        <v>0.9513</v>
       </c>
       <c r="C7" t="n">
-        <v>0.23869</v>
+        <v>0.12673</v>
       </c>
       <c r="D7" t="n">
-        <v>0.14995</v>
+        <v>0.11785</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.00432</v>
+        <v>0.00318</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.06633</v>
+        <v>-0.02262</v>
       </c>
       <c r="G7" t="n">
-        <v>0.06227</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.05955</v>
+        <v>0.0222</v>
       </c>
     </row>
     <row r="8">
@@ -645,25 +622,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.88392</v>
+        <v>0.89986</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2188</v>
+        <v>0.09926</v>
       </c>
       <c r="D8" t="n">
-        <v>0.11364</v>
+        <v>0.09200999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.08599999999999999</v>
+        <v>-0.07323</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.00452</v>
+        <v>0.01836</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.03785</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.08073</v>
+        <v>0.01166</v>
       </c>
     </row>
     <row r="9">
@@ -673,25 +647,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.45809</v>
+        <v>0.41372</v>
       </c>
       <c r="C9" t="n">
-        <v>0.26549</v>
+        <v>0.14001</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02096</v>
+        <v>0.02361</v>
       </c>
       <c r="E9" t="n">
-        <v>0.06087</v>
+        <v>0.0359</v>
       </c>
       <c r="F9" t="n">
-        <v>0.75101</v>
+        <v>0.80393</v>
       </c>
       <c r="G9" t="n">
-        <v>0.03202</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.11418</v>
+        <v>0.04855</v>
       </c>
     </row>
     <row r="10">
@@ -701,25 +672,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.37901</v>
+        <v>0.39334</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.02073</v>
+        <v>0.08371000000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>0.80371</v>
+        <v>0.76805</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01616</v>
+        <v>0.03688</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.32452</v>
+        <v>-0.38194</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.00844</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.05688</v>
+        <v>-0.00151</v>
       </c>
     </row>
     <row r="11">
@@ -729,25 +697,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.88649</v>
+        <v>0.87066</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.00235</v>
+        <v>-0.16946</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.02257</v>
+        <v>-0.01871</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.06875000000000001</v>
+        <v>-0.07076</v>
       </c>
       <c r="F11" t="n">
-        <v>0.14494</v>
+        <v>0.12402</v>
       </c>
       <c r="G11" t="n">
-        <v>0.06142</v>
-      </c>
-      <c r="H11" t="n">
-        <v>-0.01735</v>
+        <v>-0.04182</v>
       </c>
     </row>
     <row r="12">
@@ -757,25 +722,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.8364</v>
+        <v>0.77562</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.30305</v>
+        <v>-0.46046</v>
       </c>
       <c r="D12" t="n">
-        <v>0.00486</v>
+        <v>0.02119</v>
       </c>
       <c r="E12" t="n">
-        <v>0.16654</v>
+        <v>0.15435</v>
       </c>
       <c r="F12" t="n">
-        <v>0.15234</v>
+        <v>0.0438</v>
       </c>
       <c r="G12" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="H12" t="n">
-        <v>-0.06104</v>
+        <v>-0.07514</v>
       </c>
     </row>
     <row r="13">
@@ -785,25 +747,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.73872</v>
+        <v>0.73578</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.08771</v>
+        <v>-0.20005</v>
       </c>
       <c r="D13" t="n">
-        <v>0.42226</v>
+        <v>0.42493</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0595</v>
+        <v>0.05154</v>
       </c>
       <c r="F13" t="n">
-        <v>0.17655</v>
+        <v>0.11096</v>
       </c>
       <c r="G13" t="n">
-        <v>0.10712</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.05802</v>
+        <v>0.05862</v>
       </c>
     </row>
     <row r="14">
@@ -813,25 +772,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.18155</v>
+        <v>0.19054</v>
       </c>
       <c r="C14" t="n">
-        <v>0.05407</v>
+        <v>0.01448</v>
       </c>
       <c r="D14" t="n">
-        <v>0.02379</v>
+        <v>0.01487</v>
       </c>
       <c r="E14" t="n">
-        <v>0.93557</v>
+        <v>0.94443</v>
       </c>
       <c r="F14" t="n">
-        <v>0.009639999999999999</v>
+        <v>0.01223</v>
       </c>
       <c r="G14" t="n">
-        <v>0.00945</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.13018</v>
+        <v>0.11002</v>
       </c>
     </row>
     <row r="15">
@@ -841,25 +797,22 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.63845</v>
+        <v>0.59374</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.16221</v>
+        <v>-0.38343</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.12232</v>
+        <v>-0.09322</v>
       </c>
       <c r="E15" t="n">
-        <v>0.40123</v>
+        <v>0.36757</v>
       </c>
       <c r="F15" t="n">
-        <v>0.23848</v>
+        <v>0.25149</v>
       </c>
       <c r="G15" t="n">
-        <v>0.07886</v>
-      </c>
-      <c r="H15" t="n">
-        <v>-0.2318</v>
+        <v>-0.15787</v>
       </c>
     </row>
     <row r="16">
@@ -869,25 +822,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.31453</v>
+        <v>0.33917</v>
       </c>
       <c r="C16" t="n">
-        <v>0.10974</v>
+        <v>-0.01763</v>
       </c>
       <c r="D16" t="n">
-        <v>0.78993</v>
+        <v>0.80928</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.01343</v>
+        <v>-0.0294</v>
       </c>
       <c r="F16" t="n">
-        <v>0.35346</v>
+        <v>0.29891</v>
       </c>
       <c r="G16" t="n">
-        <v>0.05095</v>
-      </c>
-      <c r="H16" t="n">
-        <v>-0.01497</v>
+        <v>0.0364</v>
       </c>
     </row>
     <row r="17">
@@ -897,25 +847,22 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.25156</v>
+        <v>0.29776</v>
       </c>
       <c r="C17" t="n">
-        <v>0.14619</v>
+        <v>0.09422</v>
       </c>
       <c r="D17" t="n">
-        <v>0.02867</v>
+        <v>0.01995</v>
       </c>
       <c r="E17" t="n">
-        <v>0.11066</v>
+        <v>0.0965</v>
       </c>
       <c r="F17" t="n">
-        <v>0.05684</v>
+        <v>0.04665</v>
       </c>
       <c r="G17" t="n">
-        <v>0.09544</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.9251200000000001</v>
+        <v>0.92987</v>
       </c>
     </row>
     <row r="18">
@@ -925,25 +872,22 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6.54072</v>
+        <v>7.19247</v>
       </c>
       <c r="C18" t="n">
-        <v>1.60362</v>
+        <v>1.3524</v>
       </c>
       <c r="D18" t="n">
-        <v>1.64219</v>
+        <v>1.55675</v>
       </c>
       <c r="E18" t="n">
-        <v>1.12638</v>
+        <v>1.11185</v>
       </c>
       <c r="F18" t="n">
-        <v>1.18903</v>
+        <v>1.35711</v>
       </c>
       <c r="G18" t="n">
-        <v>0.79802</v>
-      </c>
-      <c r="H18" t="n">
-        <v>1.18391</v>
+        <v>1.16086</v>
       </c>
     </row>
     <row r="19">
@@ -953,25 +897,22 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.4088</v>
+        <v>0.44953</v>
       </c>
       <c r="C19" t="n">
-        <v>0.10023</v>
+        <v>0.08452</v>
       </c>
       <c r="D19" t="n">
-        <v>0.10264</v>
+        <v>0.0973</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0704</v>
+        <v>0.06949</v>
       </c>
       <c r="F19" t="n">
-        <v>0.07431</v>
+        <v>0.08482000000000001</v>
       </c>
       <c r="G19" t="n">
-        <v>0.04988</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.07399</v>
+        <v>0.07255</v>
       </c>
     </row>
     <row r="20">
@@ -981,25 +922,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.4088</v>
+        <v>0.44953</v>
       </c>
       <c r="C20" t="n">
-        <v>0.50902</v>
+        <v>0.53405</v>
       </c>
       <c r="D20" t="n">
-        <v>0.61166</v>
+        <v>0.63135</v>
       </c>
       <c r="E20" t="n">
-        <v>0.68206</v>
+        <v>0.70084</v>
       </c>
       <c r="F20" t="n">
-        <v>0.75637</v>
+        <v>0.78566</v>
       </c>
       <c r="G20" t="n">
-        <v>0.80625</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.88024</v>
+        <v>0.85821</v>
       </c>
     </row>
   </sheetData>

</xml_diff>